<commit_message>
Update dim_qn_variables.xlsx with new data revisions
</commit_message>
<xml_diff>
--- a/data/cs1/dim_qn_variables.xlsx
+++ b/data/cs1/dim_qn_variables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bd4428830306c10d/Documents/GitHub/DASA-Design/PyDASA-Case-Studies/data/cs1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="564" documentId="8_{E8B7102A-4272-463D-B1FF-2433195FA3DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3BB3AB2-58AD-4DC3-8BD9-413FF5495A3B}"/>
+  <xr:revisionPtr revIDLastSave="576" documentId="8_{E8B7102A-4272-463D-B1FF-2433195FA3DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3104214-0134-42D0-BCA7-948D296C4D0A}"/>
   <bookViews>
-    <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="15466" xr2:uid="{EABAE1E3-9871-4CDD-80AF-2EA34DC987B5}"/>
+    <workbookView xWindow="3140" yWindow="3140" windowWidth="19200" windowHeight="11180" xr2:uid="{EABAE1E3-9871-4CDD-80AF-2EA34DC987B5}"/>
   </bookViews>
   <sheets>
     <sheet name="dim_qn_variables" sheetId="1" r:id="rId1"/>
@@ -1382,8 +1382,8 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="str">
-        <f>_xlfn.CONCAT("\\lambda_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\lambda_{1}</v>
+        <f>_xlfn.CONCAT("\lambda_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\lambda_{1}</v>
       </c>
       <c r="D2" s="1" t="str">
         <f>_xlfn.CONCAT("lambda_tas_", Table1[[#This Row],[dm]])</f>
@@ -1453,8 +1453,8 @@
         <v>1</v>
       </c>
       <c r="C3" s="1" t="str">
-        <f>_xlfn.CONCAT("\\chi_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\chi_{1}</v>
+        <f>_xlfn.CONCAT("\chi_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\chi_{1}</v>
       </c>
       <c r="D3" s="1" t="str">
         <f>_xlfn.CONCAT("chi_tas_", Table1[[#This Row],[dm]])</f>
@@ -1524,8 +1524,8 @@
         <v>1</v>
       </c>
       <c r="C4" s="1" t="str">
-        <f>_xlfn.CONCAT("\\mu_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\mu_{1}</v>
+        <f>_xlfn.CONCAT("\mu_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\mu_{1}</v>
       </c>
       <c r="D4" s="1" t="str">
         <f>_xlfn.CONCAT("mu_tas_", Table1[[#This Row],[dm]])</f>
@@ -1654,8 +1654,8 @@
         <v>31</v>
       </c>
       <c r="T5" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1}</v>
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.5">
@@ -1796,8 +1796,8 @@
         <v>31</v>
       </c>
       <c r="T7" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.5">
@@ -1867,8 +1867,8 @@
         <v>31</v>
       </c>
       <c r="T8" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.5">
@@ -1938,8 +1938,8 @@
         <v>31</v>
       </c>
       <c r="T9" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.5">
@@ -2009,8 +2009,8 @@
         <v>31</v>
       </c>
       <c r="T10" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.0018018018018018}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.0018018018018018}</v>
       </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.5">
@@ -2080,8 +2080,8 @@
         <v>31</v>
       </c>
       <c r="T11" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.00069069069069069}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.00069069069069069}</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.5">
@@ -2092,8 +2092,8 @@
         <v>1</v>
       </c>
       <c r="C12" s="1" t="str">
-        <f>_xlfn.CONCAT("\\delta_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\delta_{1}</v>
+        <f>_xlfn.CONCAT("\delta_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\delta_{1}</v>
       </c>
       <c r="D12" s="1" t="str">
         <f>_xlfn.CONCAT("delta_tas_", Table1[[#This Row],[dm]])</f>
@@ -2151,8 +2151,8 @@
         <v>31</v>
       </c>
       <c r="T12" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 131072000', high': 1024000000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 131072000, 'high': 1024000000}</v>
       </c>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.5">
@@ -2164,8 +2164,8 @@
         <v>2</v>
       </c>
       <c r="C13" s="1" t="str">
-        <f>_xlfn.CONCAT("\\lambda_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\lambda_{2}</v>
+        <f>_xlfn.CONCAT("\lambda_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\lambda_{2}</v>
       </c>
       <c r="D13" s="1" t="str">
         <f>_xlfn.CONCAT("lambda_tas_", Table1[[#This Row],[dm]])</f>
@@ -2241,8 +2241,8 @@
         <v>2</v>
       </c>
       <c r="C14" s="1" t="str">
-        <f>_xlfn.CONCAT("\\chi_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\chi_{2}</v>
+        <f>_xlfn.CONCAT("\chi_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\chi_{2}</v>
       </c>
       <c r="D14" s="1" t="str">
         <f>_xlfn.CONCAT("chi_tas_", Table1[[#This Row],[dm]])</f>
@@ -2318,8 +2318,8 @@
         <v>2</v>
       </c>
       <c r="C15" s="1" t="str">
-        <f>_xlfn.CONCAT("\\mu_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\mu_{2}</v>
+        <f>_xlfn.CONCAT("\mu_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\mu_{2}</v>
       </c>
       <c r="D15" s="1" t="str">
         <f>_xlfn.CONCAT("mu_tas_", Table1[[#This Row],[dm]])</f>
@@ -2459,8 +2459,8 @@
         <v>uniform</v>
       </c>
       <c r="T16" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1}</v>
       </c>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.5">
@@ -2613,8 +2613,8 @@
         <v>uniform</v>
       </c>
       <c r="T18" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.5">
@@ -2690,8 +2690,8 @@
         <v>uniform</v>
       </c>
       <c r="T19" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.5">
@@ -2767,8 +2767,8 @@
         <v>uniform</v>
       </c>
       <c r="T20" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.5">
@@ -2844,8 +2844,8 @@
         <v>uniform</v>
       </c>
       <c r="T21" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.00226628895184136}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.00226628895184136}</v>
       </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.5">
@@ -2921,8 +2921,8 @@
         <v>uniform</v>
       </c>
       <c r="T22" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.000837717523269931}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.000837717523269931}</v>
       </c>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.5">
@@ -2934,8 +2934,8 @@
         <v>2</v>
       </c>
       <c r="C23" s="1" t="str">
-        <f>_xlfn.CONCAT("\\delta_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\delta_{2}</v>
+        <f>_xlfn.CONCAT("\delta_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\delta_{2}</v>
       </c>
       <c r="D23" s="1" t="str">
         <f>_xlfn.CONCAT("delta_tas_", Table1[[#This Row],[dm]])</f>
@@ -2965,7 +2965,7 @@
         <v>D*E^-1</v>
       </c>
       <c r="K23" s="1" t="str">
-        <f t="shared" ref="I23:K77" si="6">K13</f>
+        <f t="shared" ref="K23:K77" si="6">K13</f>
         <v>req/s</v>
       </c>
       <c r="L23" s="1">
@@ -2999,8 +2999,8 @@
         <v>uniform</v>
       </c>
       <c r="T23" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 131072000', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 131072000, 'high': 1000}</v>
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.5">
@@ -3012,8 +3012,8 @@
         <v>3</v>
       </c>
       <c r="C24" s="1" t="str">
-        <f>_xlfn.CONCAT("\\lambda_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\lambda_{3}</v>
+        <f>_xlfn.CONCAT("\lambda_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\lambda_{3}</v>
       </c>
       <c r="D24" s="1" t="str">
         <f>_xlfn.CONCAT("lambda_tas_", Table1[[#This Row],[dm]])</f>
@@ -3089,8 +3089,8 @@
         <v>3</v>
       </c>
       <c r="C25" s="1" t="str">
-        <f>_xlfn.CONCAT("\\chi_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\chi_{3}</v>
+        <f>_xlfn.CONCAT("\chi_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\chi_{3}</v>
       </c>
       <c r="D25" s="1" t="str">
         <f>_xlfn.CONCAT("chi_tas_", Table1[[#This Row],[dm]])</f>
@@ -3166,8 +3166,8 @@
         <v>3</v>
       </c>
       <c r="C26" s="1" t="str">
-        <f>_xlfn.CONCAT("\\mu_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\mu_{3}</v>
+        <f>_xlfn.CONCAT("\mu_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\mu_{3}</v>
       </c>
       <c r="D26" s="1" t="str">
         <f>_xlfn.CONCAT("mu_tas_", Table1[[#This Row],[dm]])</f>
@@ -3307,8 +3307,8 @@
         <v>uniform</v>
       </c>
       <c r="T27" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1}</v>
       </c>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.5">
@@ -3461,8 +3461,8 @@
         <v>uniform</v>
       </c>
       <c r="T29" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.5">
@@ -3538,8 +3538,8 @@
         <v>uniform</v>
       </c>
       <c r="T30" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="31" spans="1:20" x14ac:dyDescent="0.5">
@@ -3615,8 +3615,8 @@
         <v>uniform</v>
       </c>
       <c r="T31" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="32" spans="1:20" x14ac:dyDescent="0.5">
@@ -3692,8 +3692,8 @@
         <v>uniform</v>
       </c>
       <c r="T32" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.00189877714005237}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.00189877714005237}</v>
       </c>
     </row>
     <row r="33" spans="1:20" x14ac:dyDescent="0.5">
@@ -3769,8 +3769,8 @@
         <v>uniform</v>
       </c>
       <c r="T33" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.000470205711480949}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.000470205711480949}</v>
       </c>
     </row>
     <row r="34" spans="1:20" x14ac:dyDescent="0.5">
@@ -3782,8 +3782,8 @@
         <v>3</v>
       </c>
       <c r="C34" s="1" t="str">
-        <f>_xlfn.CONCAT("\\delta_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\delta_{3}</v>
+        <f>_xlfn.CONCAT("\delta_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\delta_{3}</v>
       </c>
       <c r="D34" s="1" t="str">
         <f>_xlfn.CONCAT("delta_tas_", Table1[[#This Row],[dm]])</f>
@@ -3847,8 +3847,8 @@
         <v>uniform</v>
       </c>
       <c r="T34" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 131072000', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 131072000, 'high': 1000}</v>
       </c>
     </row>
     <row r="35" spans="1:20" x14ac:dyDescent="0.5">
@@ -3860,8 +3860,8 @@
         <v>4</v>
       </c>
       <c r="C35" s="1" t="str">
-        <f>_xlfn.CONCAT("\\lambda_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\lambda_{4}</v>
+        <f>_xlfn.CONCAT("\lambda_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\lambda_{4}</v>
       </c>
       <c r="D35" s="1" t="str">
         <f>_xlfn.CONCAT("lambda_tas_", Table1[[#This Row],[dm]])</f>
@@ -3937,8 +3937,8 @@
         <v>4</v>
       </c>
       <c r="C36" s="1" t="str">
-        <f>_xlfn.CONCAT("\\chi_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\chi_{4}</v>
+        <f>_xlfn.CONCAT("\chi_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\chi_{4}</v>
       </c>
       <c r="D36" s="1" t="str">
         <f>_xlfn.CONCAT("chi_tas_", Table1[[#This Row],[dm]])</f>
@@ -4014,8 +4014,8 @@
         <v>4</v>
       </c>
       <c r="C37" s="1" t="str">
-        <f>_xlfn.CONCAT("\\mu_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\mu_{4}</v>
+        <f>_xlfn.CONCAT("\mu_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\mu_{4}</v>
       </c>
       <c r="D37" s="1" t="str">
         <f>_xlfn.CONCAT("mu_tas_", Table1[[#This Row],[dm]])</f>
@@ -4155,8 +4155,8 @@
         <v>uniform</v>
       </c>
       <c r="T38" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1}</v>
       </c>
     </row>
     <row r="39" spans="1:20" x14ac:dyDescent="0.5">
@@ -4309,8 +4309,8 @@
         <v>uniform</v>
       </c>
       <c r="T40" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="41" spans="1:20" x14ac:dyDescent="0.5">
@@ -4386,8 +4386,8 @@
         <v>uniform</v>
       </c>
       <c r="T41" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="42" spans="1:20" x14ac:dyDescent="0.5">
@@ -4463,8 +4463,8 @@
         <v>uniform</v>
       </c>
       <c r="T42" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="43" spans="1:20" x14ac:dyDescent="0.5">
@@ -4540,8 +4540,8 @@
         <v>uniform</v>
       </c>
       <c r="T43" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.0120527306967984}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.0120527306967984}</v>
       </c>
     </row>
     <row r="44" spans="1:20" x14ac:dyDescent="0.5">
@@ -4617,8 +4617,8 @@
         <v>uniform</v>
       </c>
       <c r="T44" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.00649717514124293}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.00649717514124293}</v>
       </c>
     </row>
     <row r="45" spans="1:20" x14ac:dyDescent="0.5">
@@ -4630,8 +4630,8 @@
         <v>4</v>
       </c>
       <c r="C45" s="1" t="str">
-        <f>_xlfn.CONCAT("\\delta_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\delta_{4}</v>
+        <f>_xlfn.CONCAT("\delta_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\delta_{4}</v>
       </c>
       <c r="D45" s="1" t="str">
         <f>_xlfn.CONCAT("delta_tas_", Table1[[#This Row],[dm]])</f>
@@ -4695,8 +4695,8 @@
         <v>uniform</v>
       </c>
       <c r="T45" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 131072000', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 131072000, 'high': 1000}</v>
       </c>
     </row>
     <row r="46" spans="1:20" x14ac:dyDescent="0.5">
@@ -4708,8 +4708,8 @@
         <v>5</v>
       </c>
       <c r="C46" s="1" t="str">
-        <f>_xlfn.CONCAT("\\lambda_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\lambda_{5}</v>
+        <f>_xlfn.CONCAT("\lambda_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\lambda_{5}</v>
       </c>
       <c r="D46" s="1" t="str">
         <f>_xlfn.CONCAT("lambda_tas_", Table1[[#This Row],[dm]])</f>
@@ -4785,8 +4785,8 @@
         <v>5</v>
       </c>
       <c r="C47" s="1" t="str">
-        <f>_xlfn.CONCAT("\\chi_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\chi_{5}</v>
+        <f>_xlfn.CONCAT("\chi_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\chi_{5}</v>
       </c>
       <c r="D47" s="1" t="str">
         <f>_xlfn.CONCAT("chi_tas_", Table1[[#This Row],[dm]])</f>
@@ -4862,8 +4862,8 @@
         <v>5</v>
       </c>
       <c r="C48" s="1" t="str">
-        <f>_xlfn.CONCAT("\\mu_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\mu_{5}</v>
+        <f>_xlfn.CONCAT("\mu_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\mu_{5}</v>
       </c>
       <c r="D48" s="1" t="str">
         <f>_xlfn.CONCAT("mu_tas_", Table1[[#This Row],[dm]])</f>
@@ -5003,8 +5003,8 @@
         <v>uniform</v>
       </c>
       <c r="T49" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1}</v>
       </c>
     </row>
     <row r="50" spans="1:20" x14ac:dyDescent="0.5">
@@ -5157,8 +5157,8 @@
         <v>uniform</v>
       </c>
       <c r="T51" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="52" spans="1:20" x14ac:dyDescent="0.5">
@@ -5234,8 +5234,8 @@
         <v>uniform</v>
       </c>
       <c r="T52" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="53" spans="1:20" x14ac:dyDescent="0.5">
@@ -5311,8 +5311,8 @@
         <v>uniform</v>
       </c>
       <c r="T53" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="54" spans="1:20" x14ac:dyDescent="0.5">
@@ -5388,8 +5388,8 @@
         <v>uniform</v>
       </c>
       <c r="T54" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.00228213858470599}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.00228213858470599}</v>
       </c>
     </row>
     <row r="55" spans="1:20" x14ac:dyDescent="0.5">
@@ -5465,8 +5465,8 @@
         <v>uniform</v>
       </c>
       <c r="T55" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.000395346131875801}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.000395346131875801}</v>
       </c>
     </row>
     <row r="56" spans="1:20" x14ac:dyDescent="0.5">
@@ -5478,8 +5478,8 @@
         <v>5</v>
       </c>
       <c r="C56" s="1" t="str">
-        <f>_xlfn.CONCAT("\\delta_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\delta_{5}</v>
+        <f>_xlfn.CONCAT("\delta_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\delta_{5}</v>
       </c>
       <c r="D56" s="1" t="str">
         <f>_xlfn.CONCAT("delta_tas_", Table1[[#This Row],[dm]])</f>
@@ -5543,8 +5543,8 @@
         <v>uniform</v>
       </c>
       <c r="T56" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 131072000', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 131072000, 'high': 1000}</v>
       </c>
     </row>
     <row r="57" spans="1:20" x14ac:dyDescent="0.5">
@@ -5556,8 +5556,8 @@
         <v>6</v>
       </c>
       <c r="C57" s="1" t="str">
-        <f>_xlfn.CONCAT("\\lambda_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\lambda_{6}</v>
+        <f>_xlfn.CONCAT("\lambda_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\lambda_{6}</v>
       </c>
       <c r="D57" s="1" t="str">
         <f>_xlfn.CONCAT("lambda_tas_", Table1[[#This Row],[dm]])</f>
@@ -5633,8 +5633,8 @@
         <v>6</v>
       </c>
       <c r="C58" s="1" t="str">
-        <f>_xlfn.CONCAT("\\chi_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\chi_{6}</v>
+        <f>_xlfn.CONCAT("\chi_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\chi_{6}</v>
       </c>
       <c r="D58" s="1" t="str">
         <f>_xlfn.CONCAT("chi_tas_", Table1[[#This Row],[dm]])</f>
@@ -5710,8 +5710,8 @@
         <v>6</v>
       </c>
       <c r="C59" s="1" t="str">
-        <f>_xlfn.CONCAT("\\mu_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\mu_{6}</v>
+        <f>_xlfn.CONCAT("\mu_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\mu_{6}</v>
       </c>
       <c r="D59" s="1" t="str">
         <f>_xlfn.CONCAT("mu_tas_", Table1[[#This Row],[dm]])</f>
@@ -5851,8 +5851,8 @@
         <v>uniform</v>
       </c>
       <c r="T60" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1}</v>
       </c>
     </row>
     <row r="61" spans="1:20" x14ac:dyDescent="0.5">
@@ -6005,8 +6005,8 @@
         <v>uniform</v>
       </c>
       <c r="T62" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="63" spans="1:20" x14ac:dyDescent="0.5">
@@ -6082,8 +6082,8 @@
         <v>uniform</v>
       </c>
       <c r="T63" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="64" spans="1:20" x14ac:dyDescent="0.5">
@@ -6159,8 +6159,8 @@
         <v>uniform</v>
       </c>
       <c r="T64" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="65" spans="1:20" x14ac:dyDescent="0.5">
@@ -6236,8 +6236,8 @@
         <v>uniform</v>
       </c>
       <c r="T65" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.0218012628780325}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.0218012628780325}</v>
       </c>
     </row>
     <row r="66" spans="1:20" x14ac:dyDescent="0.5">
@@ -6313,8 +6313,8 @@
         <v>uniform</v>
       </c>
       <c r="T66" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.0151345962113659}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.0151345962113659}</v>
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.5">
@@ -6326,8 +6326,8 @@
         <v>6</v>
       </c>
       <c r="C67" s="1" t="str">
-        <f>_xlfn.CONCAT("\\delta_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\delta_{6}</v>
+        <f>_xlfn.CONCAT("\delta_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\delta_{6}</v>
       </c>
       <c r="D67" s="1" t="str">
         <f>_xlfn.CONCAT("delta_tas_", Table1[[#This Row],[dm]])</f>
@@ -6391,8 +6391,8 @@
         <v>uniform</v>
       </c>
       <c r="T67" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 131072000', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 131072000, 'high': 1000}</v>
       </c>
     </row>
     <row r="68" spans="1:20" x14ac:dyDescent="0.5">
@@ -6404,8 +6404,8 @@
         <v>7</v>
       </c>
       <c r="C68" s="1" t="str">
-        <f>_xlfn.CONCAT("\\lambda_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\lambda_{7}</v>
+        <f>_xlfn.CONCAT("\lambda_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\lambda_{7}</v>
       </c>
       <c r="D68" s="1" t="str">
         <f>_xlfn.CONCAT("lambda_tas_", Table1[[#This Row],[dm]])</f>
@@ -6481,8 +6481,8 @@
         <v>7</v>
       </c>
       <c r="C69" s="1" t="str">
-        <f>_xlfn.CONCAT("\\chi_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\chi_{7}</v>
+        <f>_xlfn.CONCAT("\chi_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\chi_{7}</v>
       </c>
       <c r="D69" s="1" t="str">
         <f>_xlfn.CONCAT("chi_tas_", Table1[[#This Row],[dm]])</f>
@@ -6558,8 +6558,8 @@
         <v>7</v>
       </c>
       <c r="C70" s="1" t="str">
-        <f>_xlfn.CONCAT("\\mu_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\mu_{7}</v>
+        <f>_xlfn.CONCAT("\mu_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\mu_{7}</v>
       </c>
       <c r="D70" s="1" t="str">
         <f>_xlfn.CONCAT("mu_tas_", Table1[[#This Row],[dm]])</f>
@@ -6699,8 +6699,8 @@
         <v>uniform</v>
       </c>
       <c r="T71" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1}</v>
       </c>
     </row>
     <row r="72" spans="1:20" x14ac:dyDescent="0.5">
@@ -6853,8 +6853,8 @@
         <v>uniform</v>
       </c>
       <c r="T73" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="74" spans="1:20" x14ac:dyDescent="0.5">
@@ -6930,8 +6930,8 @@
         <v>uniform</v>
       </c>
       <c r="T74" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="75" spans="1:20" x14ac:dyDescent="0.5">
@@ -7007,8 +7007,8 @@
         <v>uniform</v>
       </c>
       <c r="T75" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="76" spans="1:20" x14ac:dyDescent="0.5">
@@ -7084,8 +7084,8 @@
         <v>uniform</v>
       </c>
       <c r="T76" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.00157300492372192}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.00157300492372192}</v>
       </c>
     </row>
     <row r="77" spans="1:20" x14ac:dyDescent="0.5">
@@ -7161,8 +7161,8 @@
         <v>uniform</v>
       </c>
       <c r="T77" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.000144433495150492}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.000144433495150492}</v>
       </c>
     </row>
     <row r="78" spans="1:20" x14ac:dyDescent="0.5">
@@ -7174,8 +7174,8 @@
         <v>7</v>
       </c>
       <c r="C78" s="1" t="str">
-        <f>_xlfn.CONCAT("\\delta_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\delta_{7}</v>
+        <f>_xlfn.CONCAT("\delta_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\delta_{7}</v>
       </c>
       <c r="D78" s="1" t="str">
         <f>_xlfn.CONCAT("delta_tas_", Table1[[#This Row],[dm]])</f>
@@ -7205,7 +7205,7 @@
         <v>D*E^-1</v>
       </c>
       <c r="K78" s="1" t="str">
-        <f t="shared" ref="I78:K120" si="11">K68</f>
+        <f t="shared" ref="K78:K120" si="11">K68</f>
         <v>req</v>
       </c>
       <c r="L78" s="1">
@@ -7239,8 +7239,8 @@
         <v>uniform</v>
       </c>
       <c r="T78" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 131072000', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 131072000, 'high': 1000}</v>
       </c>
     </row>
     <row r="79" spans="1:20" x14ac:dyDescent="0.5">
@@ -7252,8 +7252,8 @@
         <v>8</v>
       </c>
       <c r="C79" s="1" t="str">
-        <f>_xlfn.CONCAT("\\lambda_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\lambda_{8}</v>
+        <f>_xlfn.CONCAT("\lambda_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\lambda_{8}</v>
       </c>
       <c r="D79" s="1" t="str">
         <f>_xlfn.CONCAT("lambda_tas_", Table1[[#This Row],[dm]])</f>
@@ -7329,8 +7329,8 @@
         <v>8</v>
       </c>
       <c r="C80" s="1" t="str">
-        <f>_xlfn.CONCAT("\\chi_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\chi_{8}</v>
+        <f>_xlfn.CONCAT("\chi_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\chi_{8}</v>
       </c>
       <c r="D80" s="1" t="str">
         <f>_xlfn.CONCAT("chi_tas_", Table1[[#This Row],[dm]])</f>
@@ -7406,8 +7406,8 @@
         <v>8</v>
       </c>
       <c r="C81" s="1" t="str">
-        <f>_xlfn.CONCAT("\\mu_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\mu_{8}</v>
+        <f>_xlfn.CONCAT("\mu_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\mu_{8}</v>
       </c>
       <c r="D81" s="1" t="str">
         <f>_xlfn.CONCAT("mu_tas_", Table1[[#This Row],[dm]])</f>
@@ -7547,8 +7547,8 @@
         <v>uniform</v>
       </c>
       <c r="T82" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1}</v>
       </c>
     </row>
     <row r="83" spans="1:20" x14ac:dyDescent="0.5">
@@ -7701,8 +7701,8 @@
         <v>uniform</v>
       </c>
       <c r="T84" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="85" spans="1:20" x14ac:dyDescent="0.5">
@@ -7778,8 +7778,8 @@
         <v>uniform</v>
       </c>
       <c r="T85" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="86" spans="1:20" x14ac:dyDescent="0.5">
@@ -7855,8 +7855,8 @@
         <v>uniform</v>
       </c>
       <c r="T86" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="87" spans="1:20" x14ac:dyDescent="0.5">
@@ -7932,8 +7932,8 @@
         <v>uniform</v>
       </c>
       <c r="T87" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.00285377890156221}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.00285377890156221}</v>
       </c>
     </row>
     <row r="88" spans="1:20" x14ac:dyDescent="0.5">
@@ -8003,8 +8003,8 @@
         <v>uniform</v>
       </c>
       <c r="T88" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0}</v>
       </c>
     </row>
     <row r="89" spans="1:20" x14ac:dyDescent="0.5">
@@ -8016,8 +8016,8 @@
         <v>8</v>
       </c>
       <c r="C89" s="1" t="str">
-        <f>_xlfn.CONCAT("\\delta_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\delta_{8}</v>
+        <f>_xlfn.CONCAT("\delta_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\delta_{8}</v>
       </c>
       <c r="D89" s="1" t="str">
         <f>_xlfn.CONCAT("delta_tas_", Table1[[#This Row],[dm]])</f>
@@ -8081,8 +8081,8 @@
         <v>uniform</v>
       </c>
       <c r="T89" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 131072000', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 131072000, 'high': 1000}</v>
       </c>
     </row>
     <row r="90" spans="1:20" x14ac:dyDescent="0.5">
@@ -8094,8 +8094,8 @@
         <v>9</v>
       </c>
       <c r="C90" s="1" t="str">
-        <f>_xlfn.CONCAT("\\lambda_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\lambda_{9}</v>
+        <f>_xlfn.CONCAT("\lambda_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\lambda_{9}</v>
       </c>
       <c r="D90" s="1" t="str">
         <f>_xlfn.CONCAT("lambda_tas_", Table1[[#This Row],[dm]])</f>
@@ -8171,8 +8171,8 @@
         <v>9</v>
       </c>
       <c r="C91" s="1" t="str">
-        <f>_xlfn.CONCAT("\\chi_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\chi_{9}</v>
+        <f>_xlfn.CONCAT("\chi_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\chi_{9}</v>
       </c>
       <c r="D91" s="1" t="str">
         <f>_xlfn.CONCAT("chi_tas_", Table1[[#This Row],[dm]])</f>
@@ -8248,8 +8248,8 @@
         <v>9</v>
       </c>
       <c r="C92" s="1" t="str">
-        <f>_xlfn.CONCAT("\\mu_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\mu_{9}</v>
+        <f>_xlfn.CONCAT("\mu_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\mu_{9}</v>
       </c>
       <c r="D92" s="1" t="str">
         <f>_xlfn.CONCAT("mu_tas_", Table1[[#This Row],[dm]])</f>
@@ -8389,8 +8389,8 @@
         <v>uniform</v>
       </c>
       <c r="T93" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1}</v>
       </c>
     </row>
     <row r="94" spans="1:20" x14ac:dyDescent="0.5">
@@ -8543,8 +8543,8 @@
         <v>uniform</v>
       </c>
       <c r="T95" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="96" spans="1:20" x14ac:dyDescent="0.5">
@@ -8620,8 +8620,8 @@
         <v>uniform</v>
       </c>
       <c r="T96" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="97" spans="1:20" x14ac:dyDescent="0.5">
@@ -8697,8 +8697,8 @@
         <v>uniform</v>
       </c>
       <c r="T97" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="98" spans="1:20" x14ac:dyDescent="0.5">
@@ -8774,8 +8774,8 @@
         <v>uniform</v>
       </c>
       <c r="T98" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.000662146805468598}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.000662146805468598}</v>
       </c>
     </row>
     <row r="99" spans="1:20" x14ac:dyDescent="0.5">
@@ -8851,8 +8851,8 @@
         <v>uniform</v>
       </c>
       <c r="T99" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 2.92354130635357E-05}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 2.92354130635357E-05}</v>
       </c>
     </row>
     <row r="100" spans="1:20" x14ac:dyDescent="0.5">
@@ -8864,8 +8864,8 @@
         <v>9</v>
       </c>
       <c r="C100" s="1" t="str">
-        <f>_xlfn.CONCAT("\\delta_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\delta_{9}</v>
+        <f>_xlfn.CONCAT("\delta_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\delta_{9}</v>
       </c>
       <c r="D100" s="1" t="str">
         <f>_xlfn.CONCAT("delta_tas_", Table1[[#This Row],[dm]])</f>
@@ -8929,8 +8929,8 @@
         <v>uniform</v>
       </c>
       <c r="T100" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 131072000', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 131072000, 'high': 1000}</v>
       </c>
     </row>
     <row r="101" spans="1:20" x14ac:dyDescent="0.5">
@@ -8942,8 +8942,8 @@
         <v>10</v>
       </c>
       <c r="C101" s="1" t="str">
-        <f>_xlfn.CONCAT("\\lambda_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\lambda_{10}</v>
+        <f>_xlfn.CONCAT("\lambda_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\lambda_{10}</v>
       </c>
       <c r="D101" s="1" t="str">
         <f>_xlfn.CONCAT("lambda_tas_", Table1[[#This Row],[dm]])</f>
@@ -9019,8 +9019,8 @@
         <v>10</v>
       </c>
       <c r="C102" s="1" t="str">
-        <f>_xlfn.CONCAT("\\chi_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\chi_{10}</v>
+        <f>_xlfn.CONCAT("\chi_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\chi_{10}</v>
       </c>
       <c r="D102" s="1" t="str">
         <f>_xlfn.CONCAT("chi_tas_", Table1[[#This Row],[dm]])</f>
@@ -9096,8 +9096,8 @@
         <v>10</v>
       </c>
       <c r="C103" s="1" t="str">
-        <f>_xlfn.CONCAT("\\mu_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\mu_{10}</v>
+        <f>_xlfn.CONCAT("\mu_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\mu_{10}</v>
       </c>
       <c r="D103" s="1" t="str">
         <f>_xlfn.CONCAT("mu_tas_", Table1[[#This Row],[dm]])</f>
@@ -9237,8 +9237,8 @@
         <v>uniform</v>
       </c>
       <c r="T104" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1}</v>
       </c>
     </row>
     <row r="105" spans="1:20" x14ac:dyDescent="0.5">
@@ -9391,8 +9391,8 @@
         <v>uniform</v>
       </c>
       <c r="T106" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="107" spans="1:20" x14ac:dyDescent="0.5">
@@ -9468,8 +9468,8 @@
         <v>uniform</v>
       </c>
       <c r="T107" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="108" spans="1:20" x14ac:dyDescent="0.5">
@@ -9545,8 +9545,8 @@
         <v>uniform</v>
       </c>
       <c r="T108" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="109" spans="1:20" x14ac:dyDescent="0.5">
@@ -9622,8 +9622,8 @@
         <v>uniform</v>
       </c>
       <c r="T109" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.00225307685808432}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.00225307685808432}</v>
       </c>
     </row>
     <row r="110" spans="1:20" x14ac:dyDescent="0.5">
@@ -9699,8 +9699,8 @@
         <v>uniform</v>
       </c>
       <c r="T110" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.000824505429512892}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.000824505429512892}</v>
       </c>
     </row>
     <row r="111" spans="1:20" x14ac:dyDescent="0.5">
@@ -9712,8 +9712,8 @@
         <v>10</v>
       </c>
       <c r="C111" s="1" t="str">
-        <f>_xlfn.CONCAT("\\delta_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\delta_{10}</v>
+        <f>_xlfn.CONCAT("\delta_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\delta_{10}</v>
       </c>
       <c r="D111" s="1" t="str">
         <f>_xlfn.CONCAT("delta_tas_", Table1[[#This Row],[dm]])</f>
@@ -9777,8 +9777,8 @@
         <v>uniform</v>
       </c>
       <c r="T111" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 131072000', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 131072000, 'high': 1000}</v>
       </c>
     </row>
     <row r="112" spans="1:20" x14ac:dyDescent="0.5">
@@ -9790,8 +9790,8 @@
         <v>11</v>
       </c>
       <c r="C112" s="1" t="str">
-        <f>_xlfn.CONCAT("\\lambda_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\lambda_{11}</v>
+        <f>_xlfn.CONCAT("\lambda_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\lambda_{11}</v>
       </c>
       <c r="D112" s="1" t="str">
         <f>_xlfn.CONCAT("lambda_tas_", Table1[[#This Row],[dm]])</f>
@@ -9867,8 +9867,8 @@
         <v>11</v>
       </c>
       <c r="C113" s="1" t="str">
-        <f>_xlfn.CONCAT("\\chi_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\chi_{11}</v>
+        <f>_xlfn.CONCAT("\chi_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\chi_{11}</v>
       </c>
       <c r="D113" s="1" t="str">
         <f>_xlfn.CONCAT("chi_tas_", Table1[[#This Row],[dm]])</f>
@@ -9944,8 +9944,8 @@
         <v>11</v>
       </c>
       <c r="C114" s="1" t="str">
-        <f>_xlfn.CONCAT("\\mu_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\mu_{11}</v>
+        <f>_xlfn.CONCAT("\mu_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\mu_{11}</v>
       </c>
       <c r="D114" s="1" t="str">
         <f>_xlfn.CONCAT("mu_tas_", Table1[[#This Row],[dm]])</f>
@@ -10085,8 +10085,8 @@
         <v>uniform</v>
       </c>
       <c r="T115" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1}</v>
       </c>
     </row>
     <row r="116" spans="1:20" x14ac:dyDescent="0.5">
@@ -10239,8 +10239,8 @@
         <v>uniform</v>
       </c>
       <c r="T117" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="118" spans="1:20" x14ac:dyDescent="0.5">
@@ -10316,8 +10316,8 @@
         <v>uniform</v>
       </c>
       <c r="T118" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="119" spans="1:20" x14ac:dyDescent="0.5">
@@ -10393,8 +10393,8 @@
         <v>uniform</v>
       </c>
       <c r="T119" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="120" spans="1:20" x14ac:dyDescent="0.5">
@@ -10470,8 +10470,8 @@
         <v>uniform</v>
       </c>
       <c r="T120" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.00268792294998129}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.00268792294998129}</v>
       </c>
     </row>
     <row r="121" spans="1:20" x14ac:dyDescent="0.5">
@@ -10514,7 +10514,7 @@
         <v>T*E^-1</v>
       </c>
       <c r="K121" s="1" t="str">
-        <f t="shared" ref="I121:K132" si="14">K111</f>
+        <f t="shared" ref="K121:K132" si="14">K111</f>
         <v>s/req</v>
       </c>
       <c r="L121" s="1">
@@ -10547,8 +10547,8 @@
         <v>uniform</v>
       </c>
       <c r="T121" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.000869741131799472}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.000869741131799472}</v>
       </c>
     </row>
     <row r="122" spans="1:20" x14ac:dyDescent="0.5">
@@ -10560,8 +10560,8 @@
         <v>11</v>
       </c>
       <c r="C122" s="1" t="str">
-        <f>_xlfn.CONCAT("\\delta_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\delta_{11}</v>
+        <f>_xlfn.CONCAT("\delta_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\delta_{11}</v>
       </c>
       <c r="D122" s="1" t="str">
         <f>_xlfn.CONCAT("delta_tas_", Table1[[#This Row],[dm]])</f>
@@ -10625,8 +10625,8 @@
         <v>uniform</v>
       </c>
       <c r="T122" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 131072000', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 131072000, 'high': 1000}</v>
       </c>
     </row>
     <row r="123" spans="1:20" x14ac:dyDescent="0.5">
@@ -10638,8 +10638,8 @@
         <v>12</v>
       </c>
       <c r="C123" s="1" t="str">
-        <f>_xlfn.CONCAT("\\lambda_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\lambda_{12}</v>
+        <f>_xlfn.CONCAT("\lambda_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\lambda_{12}</v>
       </c>
       <c r="D123" s="1" t="str">
         <f>_xlfn.CONCAT("lambda_tas_", Table1[[#This Row],[dm]])</f>
@@ -10715,8 +10715,8 @@
         <v>12</v>
       </c>
       <c r="C124" s="1" t="str">
-        <f>_xlfn.CONCAT("\\chi_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\chi_{12}</v>
+        <f>_xlfn.CONCAT("\chi_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\chi_{12}</v>
       </c>
       <c r="D124" s="1" t="str">
         <f>_xlfn.CONCAT("chi_tas_", Table1[[#This Row],[dm]])</f>
@@ -10792,8 +10792,8 @@
         <v>12</v>
       </c>
       <c r="C125" s="1" t="str">
-        <f>_xlfn.CONCAT("\\mu_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\mu_{12}</v>
+        <f>_xlfn.CONCAT("\mu_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\mu_{12}</v>
       </c>
       <c r="D125" s="1" t="str">
         <f>_xlfn.CONCAT("mu_tas_", Table1[[#This Row],[dm]])</f>
@@ -10933,8 +10933,8 @@
         <v>uniform</v>
       </c>
       <c r="T126" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1}</v>
       </c>
     </row>
     <row r="127" spans="1:20" x14ac:dyDescent="0.5">
@@ -11087,8 +11087,8 @@
         <v>uniform</v>
       </c>
       <c r="T128" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="129" spans="1:20" x14ac:dyDescent="0.5">
@@ -11164,8 +11164,8 @@
         <v>uniform</v>
       </c>
       <c r="T129" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="130" spans="1:20" x14ac:dyDescent="0.5">
@@ -11241,8 +11241,8 @@
         <v>uniform</v>
       </c>
       <c r="T130" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="131" spans="1:20" x14ac:dyDescent="0.5">
@@ -11318,8 +11318,8 @@
         <v>uniform</v>
       </c>
       <c r="T131" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.00189254793212382}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.00189254793212382}</v>
       </c>
     </row>
     <row r="132" spans="1:20" x14ac:dyDescent="0.5">
@@ -11395,8 +11395,8 @@
         <v>uniform</v>
       </c>
       <c r="T132" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.000463976503552396}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.000463976503552396}</v>
       </c>
     </row>
     <row r="133" spans="1:20" x14ac:dyDescent="0.5">
@@ -11408,8 +11408,8 @@
         <v>12</v>
       </c>
       <c r="C133" s="1" t="str">
-        <f>_xlfn.CONCAT("\\delta_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\delta_{12}</v>
+        <f>_xlfn.CONCAT("\delta_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\delta_{12}</v>
       </c>
       <c r="D133" s="1" t="str">
         <f>_xlfn.CONCAT("delta_tas_", Table1[[#This Row],[dm]])</f>
@@ -11473,8 +11473,8 @@
         <v>uniform</v>
       </c>
       <c r="T133" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 131072000', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 131072000, 'high': 1000}</v>
       </c>
     </row>
     <row r="134" spans="1:20" x14ac:dyDescent="0.5">
@@ -11486,8 +11486,8 @@
         <v>13</v>
       </c>
       <c r="C134" s="1" t="str">
-        <f>_xlfn.CONCAT("\\lambda_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\lambda_{13}</v>
+        <f>_xlfn.CONCAT("\lambda_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\lambda_{13}</v>
       </c>
       <c r="D134" s="1" t="str">
         <f>_xlfn.CONCAT("lambda_tas_", Table1[[#This Row],[dm]])</f>
@@ -11563,8 +11563,8 @@
         <v>13</v>
       </c>
       <c r="C135" s="1" t="str">
-        <f>_xlfn.CONCAT("\\chi_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\chi_{13}</v>
+        <f>_xlfn.CONCAT("\chi_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\chi_{13}</v>
       </c>
       <c r="D135" s="1" t="str">
         <f>_xlfn.CONCAT("chi_tas_", Table1[[#This Row],[dm]])</f>
@@ -11640,8 +11640,8 @@
         <v>13</v>
       </c>
       <c r="C136" s="1" t="str">
-        <f>_xlfn.CONCAT("\\mu_{",Table1[[#This Row],[dm]], "}")</f>
-        <v>\\mu_{13}</v>
+        <f>_xlfn.CONCAT("\mu_{",Table1[[#This Row],[dm]], "}")</f>
+        <v>\mu_{13}</v>
       </c>
       <c r="D136" s="1" t="str">
         <f>_xlfn.CONCAT("mu_tas_", Table1[[#This Row],[dm]])</f>
@@ -11781,8 +11781,8 @@
         <v>uniform</v>
       </c>
       <c r="T137" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1}</v>
       </c>
     </row>
     <row r="138" spans="1:20" x14ac:dyDescent="0.5">
@@ -11935,8 +11935,8 @@
         <v>uniform</v>
       </c>
       <c r="T139" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="140" spans="1:20" x14ac:dyDescent="0.5">
@@ -12012,8 +12012,8 @@
         <v>uniform</v>
       </c>
       <c r="T140" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="141" spans="1:20" x14ac:dyDescent="0.5">
@@ -12056,7 +12056,7 @@
         <v>E</v>
       </c>
       <c r="K141" s="1" t="str">
-        <f t="shared" ref="I141:K144" si="17">K131</f>
+        <f t="shared" ref="K141:K144" si="17">K131</f>
         <v>s/req</v>
       </c>
       <c r="L141" s="1">
@@ -12089,8 +12089,8 @@
         <v>uniform</v>
       </c>
       <c r="T141" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 1000}</v>
       </c>
     </row>
     <row r="142" spans="1:20" x14ac:dyDescent="0.5">
@@ -12166,8 +12166,8 @@
         <v>uniform</v>
       </c>
       <c r="T142" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.0018834777097476}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.0018834777097476}</v>
       </c>
     </row>
     <row r="143" spans="1:20" x14ac:dyDescent="0.5">
@@ -12243,8 +12243,8 @@
         <v>uniform</v>
       </c>
       <c r="T143" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 0', high': 0.00045490628117618}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 0, 'high': 0.00045490628117618}</v>
       </c>
     </row>
     <row r="144" spans="1:20" x14ac:dyDescent="0.5">
@@ -12256,8 +12256,8 @@
         <v>13</v>
       </c>
       <c r="C144" s="1" t="str">
-        <f>_xlfn.CONCAT("\\delta_{", Table1[[#This Row],[dm]],"}")</f>
-        <v>\\delta_{13}</v>
+        <f>_xlfn.CONCAT("\delta_{", Table1[[#This Row],[dm]],"}")</f>
+        <v>\delta_{13}</v>
       </c>
       <c r="D144" s="1" t="str">
         <f>_xlfn.CONCAT("delta_tas_", Table1[[#This Row],[dm]])</f>
@@ -12321,8 +12321,8 @@
         <v>uniform</v>
       </c>
       <c r="T144" s="1" t="str">
-        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], "', high': ",Table1[[#This Row],[_std_max]],"}")</f>
-        <v>{'low': 131072000', high': 1000}</v>
+        <f>_xlfn.CONCAT("{'low': ", Table1[[#This Row],[_std_min]], ", 'high': ",Table1[[#This Row],[_std_max]],"}")</f>
+        <v>{'low': 131072000, 'high': 1000}</v>
       </c>
     </row>
   </sheetData>

</xml_diff>